<commit_message>
fixture 22 (weekly timesheet, UNDER_REVIEW): add condensed pattern + ungrouped data
- pattern-condensed.{csv,xlsx}: VALID condensed pattern (52 fields, 16 steps);
  extracts cleanly on both data files (2 weekly tables × 7 rows). The csv is
  semicolon-delimited to exercise the new delimiter auto-detection.
- data-ungrouped.xlsx: same sheet without the cosmetic cell merges, for testing
  that the table matcher does not depend on merges.
- pattern.xlsx / data.xlsx: work-in-progress. pattern.xlsx is still INVALID (an
  incomplete week1.day -> week1.day.date rename leaves a value/parent conflict);
  kept here because fixture 22 is UNDER_REVIEW and excluded from the test sweeps.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/22_weekly_timesheet/data.xlsx
+++ b/tests/fixtures/22_weekly_timesheet/data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E5E6A1E-D628-4C06-B84D-2928A514814A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0EDCBF9-C2E0-48FF-ABFA-BC3B35DD80D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -547,7 +547,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="46">
+  <borders count="45">
     <border>
       <left/>
       <right/>
@@ -658,21 +658,6 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="FF002CB8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF002CB8"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF002CB8"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF002CB8"/>
-      </top>
-      <bottom style="thick">
         <color rgb="FF002CB8"/>
       </bottom>
       <diagonal/>
@@ -1149,7 +1134,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
@@ -1174,13 +1159,13 @@
     <xf numFmtId="0" fontId="32" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="20" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="32" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="20" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="20" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1202,7 +1187,7 @@
     <xf numFmtId="0" fontId="36" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1211,13 +1196,13 @@
     <xf numFmtId="0" fontId="35" fillId="21" borderId="0" xfId="35" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="21" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="21" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="14" fontId="36" fillId="21" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="36" fillId="21" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1232,7 +1217,7 @@
     <xf numFmtId="0" fontId="36" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="21" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="21" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1241,154 +1226,154 @@
     <xf numFmtId="0" fontId="18" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="38" fillId="21" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="38" fillId="21" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="39" fillId="21" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="39" fillId="21" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="38" fillId="21" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="39" fillId="21" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="39" fillId="21" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="39" fillId="21" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="38" fillId="21" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="39" fillId="21" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="39" fillId="21" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="39" fillId="21" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="38" fillId="21" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="21" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="38" fillId="21" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="39" fillId="21" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="39" fillId="21" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="39" fillId="21" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="39" fillId="21" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="39" fillId="21" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="39" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="38" fillId="21" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="39" fillId="21" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="39" fillId="21" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="21" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="38" fillId="21" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="39" fillId="21" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="168" fontId="39" fillId="21" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="39" fillId="21" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="39" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="38" fillId="21" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="39" fillId="21" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="21" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="21" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="38" fillId="21" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="38" fillId="21" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="38" fillId="21" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="21" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="38" fillId="21" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="39" fillId="21" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="21" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="39" fillId="21" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="38" fillId="21" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="39" fillId="21" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="39" fillId="21" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="39" fillId="21" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="21" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="38" fillId="21" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="39" fillId="21" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="21" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="39" fillId="21" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="38" fillId="21" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="39" fillId="21" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="39" fillId="21" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="39" fillId="21" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="21" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="21" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="21" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="36" fillId="21" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="36" fillId="21" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="21" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="21" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="38" fillId="21" borderId="24" xfId="48" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="38" fillId="21" borderId="45" xfId="48" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="38" fillId="21" borderId="23" xfId="48" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="38" fillId="21" borderId="44" xfId="48" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="38" fillId="21" borderId="9" xfId="48" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="38" fillId="21" borderId="44" xfId="48" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="21" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="38" fillId="21" borderId="43" xfId="48" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="21" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="21" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="21" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="39" fillId="21" borderId="20" xfId="28" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="39" fillId="21" borderId="19" xfId="28" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="165" fontId="39" fillId="21" borderId="0" xfId="28" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="14" fontId="36" fillId="21" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="36" fillId="21" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1">
@@ -1412,28 +1397,29 @@
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" xfId="35" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" xfId="35" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="36" fillId="21" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="14" fontId="36" fillId="21" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="36" fillId="21" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="21" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="38" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="21" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="21" borderId="10" xfId="33" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="15" xfId="32" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="20" borderId="16" xfId="32" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="20" borderId="17" xfId="32" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="18" xfId="32" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="21" borderId="0" xfId="34" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1442,37 +1428,42 @@
     <xf numFmtId="0" fontId="36" fillId="21" borderId="8" xfId="34" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="165" fontId="38" fillId="21" borderId="16" xfId="29" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="38" fillId="21" borderId="17" xfId="29" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="38" fillId="21" borderId="18" xfId="29" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="21" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="21" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="21" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="21" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="21" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="21" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="35" fillId="21" borderId="0" xfId="45" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="21" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="21" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" xfId="35" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="21" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" xfId="35" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="15" xfId="33" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="16" xfId="33" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="17" xfId="33" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="20% - Accent1" xfId="1" builtinId="30" customBuiltin="1"/>
@@ -1543,6 +1534,58 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color indexed="9"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="5"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="166" formatCode="[$-409]h:mm\ AM/PM;@"/>
       <fill>
         <patternFill patternType="solid">
@@ -2587,58 +2630,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="5"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color indexed="9"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="major"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
@@ -2913,7 +2904,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6A5539C7-6614-4324-B8A3-2FCC3BF1A317}" name="Week1Time" displayName="Week1Time" ref="B9:E16" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6A5539C7-6614-4324-B8A3-2FCC3BF1A317}" name="Week1Time" displayName="Week1Time" ref="B9:E16" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
   <autoFilter ref="B9:E16" xr:uid="{E10A4982-6DC5-4879-AEB0-7CD24C647365}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2921,12 +2912,12 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{190B07CD-9F05-463A-BC91-7CBD9D46B2DC}" name="Day of week" dataDxfId="35">
+    <tableColumn id="1" xr3:uid="{190B07CD-9F05-463A-BC91-7CBD9D46B2DC}" name="Day of week" dataDxfId="37">
       <calculatedColumnFormula>B9+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{246B2CC2-2B22-4BC0-A2EC-BECFF2982E0C}" name="Time in" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{6F65ADD7-35CE-4B83-AE46-13F67FC9F37B}" name="Breaks_x000a_(minutes)" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{751BE875-F656-4BE3-A513-3CE9F2CDBAE5}" name="Time out" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{246B2CC2-2B22-4BC0-A2EC-BECFF2982E0C}" name="Time in" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{6F65ADD7-35CE-4B83-AE46-13F67FC9F37B}" name="Breaks_x000a_(minutes)" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{751BE875-F656-4BE3-A513-3CE9F2CDBAE5}" name="Time out" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TimeSheet table style" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
@@ -2938,7 +2929,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{522816F0-543F-433C-994E-34511C77A530}" name="Week1Breakdown" displayName="Week1Breakdown" ref="G9:L16" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{522816F0-543F-433C-994E-34511C77A530}" name="Week1Breakdown" displayName="Week1Breakdown" ref="G9:L16" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
   <autoFilter ref="G9:L16" xr:uid="{C7946D40-1373-4344-834A-34D082D7662E}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2948,14 +2939,14 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{6614CBB3-4212-476B-A68B-BDCD0C62C21C}" name="Total_x000a_[h]:mm" dataDxfId="29">
+    <tableColumn id="1" xr3:uid="{6614CBB3-4212-476B-A68B-BDCD0C62C21C}" name="Total_x000a_[h]:mm" dataDxfId="31">
       <calculatedColumnFormula>MROUND((IF(OR(C10="",E10=""),0,IF(E10&lt;C10,E10+1-C10,E10-C10))-D10/1440),1/1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{59BFD623-32D7-41A7-876C-DC30F237A3C1}" name="Regular_x000a_[h]:mm" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{BC5185F3-BC05-4AF9-83F5-457177271D1C}" name="Overtime_x000a_[h]:mm" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{BA9FADD4-9CD7-490B-A73D-26DFE1594B4A}" name="Sick_x000a_[h]:mm" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{262E2356-E5D2-41AD-8919-B71988181056}" name="Holiday_x000a_[h]:mm" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{FD71D99B-5969-4D1B-B038-07613CF9228E}" name="Vacation_x000a_[h]:mm" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{59BFD623-32D7-41A7-876C-DC30F237A3C1}" name="Regular_x000a_[h]:mm" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{BC5185F3-BC05-4AF9-83F5-457177271D1C}" name="Overtime_x000a_[h]:mm" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{BA9FADD4-9CD7-490B-A73D-26DFE1594B4A}" name="Sick_x000a_[h]:mm" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{262E2356-E5D2-41AD-8919-B71988181056}" name="Holiday_x000a_[h]:mm" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{FD71D99B-5969-4D1B-B038-07613CF9228E}" name="Vacation_x000a_[h]:mm" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TimeSheet table style" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
@@ -2967,7 +2958,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{195ADD69-B923-4124-BA0F-F0A87BFFAB8C}" name="RatePerHr" displayName="RatePerHr" ref="G29:L31" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22" tableBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{195ADD69-B923-4124-BA0F-F0A87BFFAB8C}" name="RatePerHr" displayName="RatePerHr" ref="G29:L31" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24" tableBorderDxfId="23">
   <autoFilter ref="G29:L31" xr:uid="{706249EA-B432-41B9-A04B-7D8A3AFA0A60}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2977,20 +2968,20 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{BD59BE1B-C83E-42A4-96F2-465DEFAB470E}" name=" " dataDxfId="20" dataCellStyle="Normal"/>
-    <tableColumn id="2" xr3:uid="{069F8AEE-8755-45F7-8979-AE6E8F82BA6E}" name="Regular" dataDxfId="19">
+    <tableColumn id="1" xr3:uid="{BD59BE1B-C83E-42A4-96F2-465DEFAB470E}" name=" " dataDxfId="22" dataCellStyle="Normal"/>
+    <tableColumn id="2" xr3:uid="{069F8AEE-8755-45F7-8979-AE6E8F82BA6E}" name="Regular" dataDxfId="21">
       <calculatedColumnFormula>ROUND((H26+H16)*24*H29,2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{226B57E1-FB02-4033-A5BE-9DA8E24BB60D}" name="Overtime" dataDxfId="18">
+    <tableColumn id="3" xr3:uid="{226B57E1-FB02-4033-A5BE-9DA8E24BB60D}" name="Overtime" dataDxfId="20">
       <calculatedColumnFormula>ROUND((I26+I16)*24*I29,2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{6EE04012-C2D5-4A70-8F77-F47EFBB2A20E}" name="Sick" dataDxfId="17">
+    <tableColumn id="4" xr3:uid="{6EE04012-C2D5-4A70-8F77-F47EFBB2A20E}" name="Sick" dataDxfId="19">
       <calculatedColumnFormula>ROUND((J26+J16)*24*J29,2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{919C7435-5B52-4BF0-A776-D8CBE5F5967A}" name="Holiday" dataDxfId="16">
+    <tableColumn id="5" xr3:uid="{919C7435-5B52-4BF0-A776-D8CBE5F5967A}" name="Holiday" dataDxfId="18">
       <calculatedColumnFormula>ROUND((K26+K16)*24*K29,2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{35FA5A78-FAF8-4870-A653-E29A9BB3A0AA}" name="Vacation" dataDxfId="15">
+    <tableColumn id="6" xr3:uid="{35FA5A78-FAF8-4870-A653-E29A9BB3A0AA}" name="Vacation" dataDxfId="17">
       <calculatedColumnFormula>ROUND((L26+L16)*24*L29,2)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3004,7 +2995,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A0AD4DFC-2CD1-4792-B7D3-DF944748F7F4}" name="Week2Breakdown" displayName="Week2Breakdown" ref="G19:L26" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A0AD4DFC-2CD1-4792-B7D3-DF944748F7F4}" name="Week2Breakdown" displayName="Week2Breakdown" ref="G19:L26" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="G19:L26" xr:uid="{A44E8DD1-E48F-486F-8ACA-EBA1479FCFE1}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3014,14 +3005,14 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{1988A15C-4BA8-4142-86FB-A6C0EE7DB363}" name="Total_x000a_[h]:mm" dataDxfId="12">
+    <tableColumn id="1" xr3:uid="{1988A15C-4BA8-4142-86FB-A6C0EE7DB363}" name="Total_x000a_[h]:mm" dataDxfId="14">
       <calculatedColumnFormula>MROUND((IF(OR(C20="",E20=""),0,IF(E20&lt;C20,E20+1-C20,E20-C20))-D20/1440),1/1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D83BC574-D19E-4A38-B74A-DBB7077A3F47}" name="Regular_x000a_[h]:mm" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{BB4E3C4E-F96F-4A73-AE63-30F72E93F87C}" name="Overtime_x000a_[h]:mm" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{D0989223-D47C-4886-A250-E68512C37A87}" name="Sick_x000a_[h]:mm" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{08B2B68A-21F4-4897-89DF-8226A098DD8A}" name="Holiday_x000a_[h]:mm" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{D2CDB383-0ABA-4980-A10D-E413B7B160E5}" name="Vacation_x000a_[h]:mm" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{D83BC574-D19E-4A38-B74A-DBB7077A3F47}" name="Regular_x000a_[h]:mm" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{BB4E3C4E-F96F-4A73-AE63-30F72E93F87C}" name="Overtime_x000a_[h]:mm" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{D0989223-D47C-4886-A250-E68512C37A87}" name="Sick_x000a_[h]:mm" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{08B2B68A-21F4-4897-89DF-8226A098DD8A}" name="Holiday_x000a_[h]:mm" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{D2CDB383-0ABA-4980-A10D-E413B7B160E5}" name="Vacation_x000a_[h]:mm" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TimeSheet table style" showFirstColumn="1" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
   <extLst>
@@ -3033,7 +3024,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A2E9F439-BCBA-433C-B159-4BAFDA05F0EF}" name="Week2Time" displayName="Week2Time" ref="B19:E26" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5" tableBorderDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A2E9F439-BCBA-433C-B159-4BAFDA05F0EF}" name="Week2Time" displayName="Week2Time" ref="B19:E26" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7" tableBorderDxfId="6">
   <autoFilter ref="B19:E26" xr:uid="{042AB274-B97B-41F5-8F67-3A0C22AE718C}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3041,12 +3032,12 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{3D04EA17-D67B-4FF5-AE8F-3C4501211381}" name="Day of week" dataDxfId="3">
+    <tableColumn id="1" xr3:uid="{3D04EA17-D67B-4FF5-AE8F-3C4501211381}" name="Day of week" dataDxfId="5">
       <calculatedColumnFormula>B19+1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{BCC6F48D-C6D2-4D1C-9C72-68418FF1D1D1}" name="Time in" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{2AB5FEA2-436C-4712-BC1F-76D8785BC4CB}" name="Breaks_x000a_(minutes)" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{7902BB71-D1CD-4EC4-BED2-0A23C5CE00F2}" name="Time out" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{BCC6F48D-C6D2-4D1C-9C72-68418FF1D1D1}" name="Time in" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{2AB5FEA2-436C-4712-BC1F-76D8785BC4CB}" name="Breaks_x000a_(minutes)" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{7902BB71-D1CD-4EC4-BED2-0A23C5CE00F2}" name="Time out" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TimeSheet table style" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
@@ -3353,21 +3344,21 @@
     </row>
     <row r="2" spans="1:15" ht="75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="5"/>
-      <c r="B2" s="93" t="s">
+      <c r="B2" s="94" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="94"/>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="92" t="s">
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="108" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="92"/>
-      <c r="I2" s="92"/>
-      <c r="J2" s="92"/>
-      <c r="K2" s="92"/>
-      <c r="L2" s="92"/>
+      <c r="H2" s="109"/>
+      <c r="I2" s="109"/>
+      <c r="J2" s="109"/>
+      <c r="K2" s="109"/>
+      <c r="L2" s="110"/>
       <c r="M2" s="5"/>
     </row>
     <row r="3" spans="1:15" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
@@ -3387,21 +3378,21 @@
     </row>
     <row r="4" spans="1:15" s="19" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="13"/>
-      <c r="B4" s="96" t="s">
+      <c r="B4" s="97" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="96"/>
-      <c r="D4" s="96"/>
+      <c r="C4" s="97"/>
+      <c r="D4" s="97"/>
       <c r="E4" s="14"/>
       <c r="F4" s="15"/>
-      <c r="G4" s="108" t="s">
+      <c r="G4" s="88" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="108"/>
-      <c r="I4" s="88" t="s">
+      <c r="H4" s="88"/>
+      <c r="I4" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="88"/>
+      <c r="J4" s="90"/>
       <c r="K4" s="16"/>
       <c r="L4" s="17"/>
       <c r="M4" s="18"/>
@@ -3417,14 +3408,14 @@
       <c r="D5" s="107"/>
       <c r="E5" s="14"/>
       <c r="F5" s="20"/>
-      <c r="G5" s="106" t="s">
+      <c r="G5" s="89" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="106"/>
-      <c r="I5" s="105" t="s">
+      <c r="H5" s="89"/>
+      <c r="I5" s="106" t="s">
         <v>18</v>
       </c>
-      <c r="J5" s="105"/>
+      <c r="J5" s="106"/>
       <c r="K5" s="21"/>
       <c r="L5" s="22"/>
       <c r="M5" s="18"/>
@@ -3432,22 +3423,22 @@
     </row>
     <row r="6" spans="1:15" s="19" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="13"/>
-      <c r="B6" s="97" t="s">
+      <c r="B6" s="98" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="97"/>
-      <c r="D6" s="97"/>
+      <c r="C6" s="98"/>
+      <c r="D6" s="98"/>
       <c r="E6" s="14"/>
       <c r="F6" s="20"/>
-      <c r="G6" s="106" t="s">
+      <c r="G6" s="89" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="106"/>
-      <c r="I6" s="89">
+      <c r="H6" s="89"/>
+      <c r="I6" s="91">
         <f ca="1">TODAY()</f>
-        <v>46183</v>
-      </c>
-      <c r="J6" s="89"/>
+        <v>46184</v>
+      </c>
+      <c r="J6" s="91"/>
       <c r="K6" s="23"/>
       <c r="L6" s="24"/>
       <c r="M6" s="13"/>
@@ -3455,11 +3446,11 @@
     </row>
     <row r="7" spans="1:15" s="19" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="13"/>
-      <c r="B7" s="104" t="s">
+      <c r="B7" s="105" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="104"/>
-      <c r="D7" s="104"/>
+      <c r="C7" s="105"/>
+      <c r="D7" s="105"/>
       <c r="E7" s="25"/>
       <c r="F7" s="24"/>
       <c r="G7" s="26"/>
@@ -3524,7 +3515,7 @@
       <c r="A10" s="13"/>
       <c r="B10" s="85">
         <f ca="1">Week_Starting</f>
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="C10" s="86">
         <v>0.37847222222222227</v>
@@ -3556,7 +3547,7 @@
       <c r="A11" s="13"/>
       <c r="B11" s="85">
         <f t="shared" ref="B11:B16" ca="1" si="0">B10+1</f>
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="C11" s="86">
         <v>0.37847222222222227</v>
@@ -3588,7 +3579,7 @@
       <c r="A12" s="13"/>
       <c r="B12" s="85">
         <f t="shared" ca="1" si="0"/>
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="C12" s="86">
         <v>0.375</v>
@@ -3619,7 +3610,7 @@
       <c r="A13" s="13"/>
       <c r="B13" s="85">
         <f t="shared" ca="1" si="0"/>
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="C13" s="86">
         <v>0.375</v>
@@ -3650,7 +3641,7 @@
       <c r="A14" s="13"/>
       <c r="B14" s="85">
         <f t="shared" ca="1" si="0"/>
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="C14" s="86"/>
       <c r="D14" s="87"/>
@@ -3673,7 +3664,7 @@
       <c r="A15" s="13"/>
       <c r="B15" s="85">
         <f t="shared" ca="1" si="0"/>
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="C15" s="86"/>
       <c r="D15" s="87"/>
@@ -3694,7 +3685,7 @@
       <c r="A16" s="13"/>
       <c r="B16" s="85">
         <f t="shared" ca="1" si="0"/>
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="C16" s="86"/>
       <c r="D16" s="87"/>
@@ -3798,7 +3789,7 @@
       <c r="A20" s="13"/>
       <c r="B20" s="31">
         <f ca="1">B16+1</f>
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="C20" s="32"/>
       <c r="D20" s="56"/>
@@ -3819,7 +3810,7 @@
       <c r="A21" s="13"/>
       <c r="B21" s="40">
         <f t="shared" ref="B21:B26" ca="1" si="2">B20+1</f>
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="C21" s="41"/>
       <c r="D21" s="43"/>
@@ -3840,7 +3831,7 @@
       <c r="A22" s="13"/>
       <c r="B22" s="49">
         <f t="shared" ca="1" si="2"/>
-        <v>46192</v>
+        <v>46193</v>
       </c>
       <c r="C22" s="41"/>
       <c r="D22" s="43"/>
@@ -3861,7 +3852,7 @@
       <c r="A23" s="13"/>
       <c r="B23" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>46193</v>
+        <v>46194</v>
       </c>
       <c r="C23" s="41"/>
       <c r="D23" s="33"/>
@@ -3882,7 +3873,7 @@
       <c r="A24" s="13"/>
       <c r="B24" s="49">
         <f t="shared" ca="1" si="2"/>
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="C24" s="42"/>
       <c r="D24" s="43"/>
@@ -3903,7 +3894,7 @@
       <c r="A25" s="13"/>
       <c r="B25" s="57">
         <f t="shared" ca="1" si="2"/>
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="C25" s="58"/>
       <c r="D25" s="59"/>
@@ -3924,7 +3915,7 @@
       <c r="A26" s="13"/>
       <c r="B26" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="C26" s="47"/>
       <c r="D26" s="33"/>
@@ -4017,9 +4008,9 @@
     </row>
     <row r="30" spans="1:14" s="19" customFormat="1" ht="35" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="13"/>
-      <c r="B30" s="102"/>
-      <c r="C30" s="102"/>
-      <c r="D30" s="102"/>
+      <c r="B30" s="103"/>
+      <c r="C30" s="103"/>
+      <c r="D30" s="103"/>
       <c r="E30" s="70"/>
       <c r="F30" s="24"/>
       <c r="G30" s="71" t="s">
@@ -4046,11 +4037,11 @@
     </row>
     <row r="31" spans="1:14" s="19" customFormat="1" ht="35" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A31" s="13"/>
-      <c r="B31" s="103" t="s">
+      <c r="B31" s="104" t="s">
         <v>7</v>
       </c>
-      <c r="C31" s="103"/>
-      <c r="D31" s="103"/>
+      <c r="C31" s="104"/>
+      <c r="D31" s="104"/>
       <c r="E31" s="76" t="s">
         <v>8</v>
       </c>
@@ -4082,9 +4073,9 @@
     </row>
     <row r="32" spans="1:14" ht="35" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="5"/>
-      <c r="B32" s="100"/>
-      <c r="C32" s="100"/>
-      <c r="D32" s="100"/>
+      <c r="B32" s="101"/>
+      <c r="C32" s="101"/>
+      <c r="D32" s="101"/>
       <c r="E32" s="80"/>
       <c r="F32" s="81"/>
       <c r="G32" s="82"/>
@@ -4097,26 +4088,26 @@
     </row>
     <row r="33" spans="1:13" ht="35" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="5"/>
-      <c r="B33" s="101" t="s">
+      <c r="B33" s="102" t="s">
         <v>9</v>
       </c>
-      <c r="C33" s="101"/>
-      <c r="D33" s="101"/>
+      <c r="C33" s="102"/>
+      <c r="D33" s="102"/>
       <c r="E33" s="24" t="s">
         <v>8</v>
       </c>
       <c r="F33" s="81"/>
-      <c r="G33" s="90" t="s">
+      <c r="G33" s="92" t="s">
         <v>17</v>
       </c>
-      <c r="H33" s="91"/>
-      <c r="I33" s="91"/>
-      <c r="J33" s="91"/>
-      <c r="K33" s="98">
+      <c r="H33" s="93"/>
+      <c r="I33" s="93"/>
+      <c r="J33" s="93"/>
+      <c r="K33" s="99">
         <f>SUM(H31:L31)</f>
         <v>652.5</v>
       </c>
-      <c r="L33" s="99"/>
+      <c r="L33" s="100"/>
       <c r="M33" s="5"/>
     </row>
     <row r="34" spans="1:13" ht="35" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
@@ -4136,11 +4127,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="G33:J33"/>
     <mergeCell ref="G2:L2"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B4:D4"/>
@@ -4154,6 +4140,11 @@
     <mergeCell ref="I5:J5"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="B5:D5"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="G33:J33"/>
   </mergeCells>
   <dataValidations count="33">
     <dataValidation type="time" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Incorrect Time Format" error="Please use the following format for entering the time: 12:00 AM" sqref="E10:E16 C10:C16 E20:E26 C20:C26" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>